<commit_message>
excel-modeling: scenarios, tornado, grid assertions, charts, render; Jordan driver ranking
xl.py scenarios flips a switch and asserts the master check, a changing output
and case ordering; tornado ranks inputs by swing; sensitivity grids now assert
odd size, centre = base, distinct cells and monotonic axes; render exports a
recalculated copy to PNG for visual review. Builder adds check templates,
source comments on every input, print setup, and live waterfall and football
field charts (stacked series, portable to LibreOffice and Sheets).

data/valuation/jordan_tornado.csv: Base-case value per NKE share is most
sensitive to the steady-state EBIT margin (8% to 14%: $2.80 to $4.79, swing
$1.99), then WACC (9% to 11%: swing $1.09), terminal growth ($0.46).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFKfBcMnBcfuRQys4LRjyK
</commit_message>
<xml_diff>
--- a/data/valuation/jordan_valuation.xlsx
+++ b/data/valuation/jordan_valuation.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Inputs" sheetId="2" r:id="rId2"/>
     <sheet name="Model" sheetId="3" r:id="rId3"/>
     <sheet name="Valuation" sheetId="4" r:id="rId4"/>
-    <sheet name="Checks" sheetId="5" r:id="rId5"/>
+    <sheet name="Charts" sheetId="5" r:id="rId5"/>
+    <sheet name="Checks" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="k_Inputs_case">Inputs!$A$5</definedName>
@@ -55,14 +56,232 @@
     <definedName name="k_Valuation_tv">Valuation!$A$6</definedName>
     <definedName name="k_Valuation_tv_share">Valuation!$A$13</definedName>
     <definedName name="k_Valuation_vs_peak">Valuation!$A$17</definedName>
-    <definedName name="MasterCheck">Checks!$D$7</definedName>
+    <definedName name="MasterCheck">Checks!$D$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">Inputs!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">Model!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">Valuation!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: FY2026 Form 10-K (filed 2026-07-15) p. 32</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: FY2026 Form 10-K (filed 2026-07-15) p. 32</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: market data, data/valuation/peer_multiples.csv (Oct 13, 2026)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C17" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: FY2027 consolidated margin implied by consensus EPS; Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Convention shared with the reverse DCF (research_notes/thesis_tests/consensus_and_valuation.md Section C)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: ASSUMPTION; see research_notes/12_jordan_brand_thesis.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: ASSUMPTION</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: ASSUMPTION; FY2027 -15% from Q1 FY27 'mid-teens' decline (Nike transcript, Oct 1, 2026)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: ASSUMPTION; FY2027 -15% from Q1 FY27 'mid-teens' decline (Nike transcript, Oct 1, 2026)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: ASSUMPTION; FY2027 -15% from Q1 FY27 'mid-teens' decline (Nike transcript, Oct 1, 2026)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="142">
   <si>
     <t>Inputs</t>
   </si>
@@ -313,6 +532,99 @@
     <t>FY2031 revenue vs FY2024 peak</t>
   </si>
   <si>
+    <t>Charts</t>
+  </si>
+  <si>
+    <t>Jordan DCF value, active scenario ($m)</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Running total</t>
+  </si>
+  <si>
+    <t>Increase</t>
+  </si>
+  <si>
+    <t>Decrease</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>PV FY2027 FCF</t>
+  </si>
+  <si>
+    <t>PV FY2028 FCF</t>
+  </si>
+  <si>
+    <t>PV FY2029 FCF</t>
+  </si>
+  <si>
+    <t>PV FY2030 FCF</t>
+  </si>
+  <si>
+    <t>PV FY2031 FCF</t>
+  </si>
+  <si>
+    <t>PV terminal value</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Live: follows the scenario switch on Inputs. End bar equals Valuation 'DCF value of Jordan'.</t>
+  </si>
+  <si>
+    <t>Jordan value per NKE share ($)</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>DCF, Bear to Bull scenarios</t>
+  </si>
+  <si>
+    <t>data/valuation/jordan_scenarios.csv (scripts/jordan_valuation.py)</t>
+  </si>
+  <si>
+    <t>DCF, Base path, margin 6% to 17%</t>
+  </si>
+  <si>
+    <t>data/valuation/jordan_sensitivity.csv</t>
+  </si>
+  <si>
+    <t>DCF, Bear path, margin 6% to 17%</t>
+  </si>
+  <si>
+    <t>Jordan FY2026 revenue x NKE EV/Sales</t>
+  </si>
+  <si>
+    <t>jordan_scenarios.csv reference row (point estimate)</t>
+  </si>
+  <si>
+    <t>Live scenario value per share</t>
+  </si>
+  <si>
+    <t>live marker (column F), drawn as a sliver of width set in column G</t>
+  </si>
+  <si>
+    <t>Static ranges are outputs of scripts/jordan_valuation.py; the marker is live.</t>
+  </si>
+  <si>
     <t>Check</t>
   </si>
   <si>
@@ -325,18 +637,24 @@
     <t>Margin reaches target in FY2031</t>
   </si>
   <si>
-    <t>WACC above terminal growth</t>
+    <t>Terminal growth below WACC</t>
   </si>
   <si>
     <t>must be 1</t>
   </si>
   <si>
+    <t>Revenue never negative</t>
+  </si>
+  <si>
     <t>Value = PV(FCF) + PV(TV)</t>
   </si>
   <si>
     <t>Discount timing ends at 4.63 years</t>
   </si>
   <si>
+    <t>Jordan DCF value, active scenario ($m): bars reconcile</t>
+  </si>
+  <si>
     <t>Master check (1 = all pass)</t>
   </si>
   <si>
@@ -386,23 +704,27 @@
   </si>
   <si>
     <t>DCF value, per-share value and terminal share for the active scenario</t>
+  </si>
+  <si>
+    <t>Value bridge for the active scenario and the per-share football field</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="@"/>
     <numFmt numFmtId="165" formatCode="#,##0_);(#,##0);&quot;-&quot;_)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00_);($#,##0.00);&quot;-&quot;_)"/>
     <numFmt numFmtId="167" formatCode="0.0%_);(0.0%);&quot;-&quot;_)"/>
     <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="#,##0.000000"/>
-    <numFmt numFmtId="171" formatCode="0.000000"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="172" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -449,6 +771,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -491,7 +819,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -517,8 +845,10 @@
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -528,6 +858,645 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Jordan DCF value, active scenario ($m)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Base</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>PV FY2027 FCF</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PV FY2028 FCF</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>PV FY2029 FCF</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>PV FY2030 FCF</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>PV FY2031 FCF</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>PV terminal value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>End</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$D$5:$D$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Total</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>PV FY2027 FCF</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PV FY2028 FCF</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>PV FY2029 FCF</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>PV FY2030 FCF</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>PV FY2031 FCF</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>PV terminal value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>End</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$G$5:$G$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Increase</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="548235"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>PV FY2027 FCF</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PV FY2028 FCF</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>PV FY2029 FCF</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>PV FY2030 FCF</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>PV FY2031 FCF</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>PV terminal value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>End</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$E$5:$E$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Decrease</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>PV FY2027 FCF</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PV FY2028 FCF</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>PV FY2029 FCF</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>PV FY2030 FCF</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>PV FY2031 FCF</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>PV terminal value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>End</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$F$5:$F$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="50"/>
+        <c:overlap val="100"/>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0_);(#,##0);&quot;-&quot;_)" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Jordan value per NKE share ($)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Low</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$38:$A$42</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>DCF, Bear to Bull scenarios</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>DCF, Base path, margin 6% to 17%</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>DCF, Bear path, margin 6% to 17%</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Jordan FY2026 revenue x NKE EV/Sales</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Live scenario value per share</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$B$38:$B$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2.32</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.68</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Range</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Charts!$A$38:$A$42</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>DCF, Bear to Bull scenarios</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>DCF, Base path, margin 6% to 17%</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>DCF, Bear path, margin 6% to 17%</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Jordan FY2026 revenue x NKE EV/Sales</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Live scenario value per share</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Charts!$D$38:$D$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="100"/>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50020001"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50020002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="t"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$#,##0.00_);($#,##0.00);&quot;-&quot;_)" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -815,7 +1784,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -824,17 +1796,17 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B4" s="1" t="str">
         <f>IF(MasterCheck=1,"OK: all checks pass","ERROR: see Checks sheet")</f>
@@ -843,44 +1815,44 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="4" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -888,7 +1860,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -896,7 +1868,7 @@
         <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -904,16 +1876,31 @@
         <v>68</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>107</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;A&amp;R&amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1197,11 +2184,19 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;A&amp;R&amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1698,11 +2693,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;A&amp;R&amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1880,12 +2883,372 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;A&amp;R&amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="38.7109375" customWidth="1"/>
+    <col min="2" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="60.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="24">
+        <f>Model!$C$22</f>
+        <v>161.47292095919</v>
+      </c>
+      <c r="C5" s="10">
+        <f>B5</f>
+        <v>161.47292095919</v>
+      </c>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10">
+        <f>B5</f>
+        <v>161.47292095919</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="24">
+        <f>Model!$D$22</f>
+        <v>283.509307261502</v>
+      </c>
+      <c r="C6" s="10">
+        <f>C5+B6</f>
+        <v>444.982228220691</v>
+      </c>
+      <c r="D6" s="10">
+        <f>MIN(C5,C6)</f>
+        <v>161.47292095919</v>
+      </c>
+      <c r="E6" s="10">
+        <f>MAX(B6,0)</f>
+        <v>283.509307261502</v>
+      </c>
+      <c r="F6" s="10">
+        <f>MAX(-B6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="24">
+        <f>Model!$E$22</f>
+        <v>226.985561882892</v>
+      </c>
+      <c r="C7" s="10">
+        <f>C6+B7</f>
+        <v>671.967790103583</v>
+      </c>
+      <c r="D7" s="10">
+        <f>MIN(C6,C7)</f>
+        <v>444.982228220691</v>
+      </c>
+      <c r="E7" s="10">
+        <f>MAX(B7,0)</f>
+        <v>226.985561882892</v>
+      </c>
+      <c r="F7" s="10">
+        <f>MAX(-B7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="10"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="24">
+        <f>Model!$F$22</f>
+        <v>265.390596257345</v>
+      </c>
+      <c r="C8" s="10">
+        <f>C7+B8</f>
+        <v>937.358386360928</v>
+      </c>
+      <c r="D8" s="10">
+        <f>MIN(C7,C8)</f>
+        <v>671.967790103583</v>
+      </c>
+      <c r="E8" s="10">
+        <f>MAX(B8,0)</f>
+        <v>265.390596257345</v>
+      </c>
+      <c r="F8" s="10">
+        <f>MAX(-B8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Model!$G$22</f>
+        <v>299.835285436841</v>
+      </c>
+      <c r="C9" s="10">
+        <f>C8+B9</f>
+        <v>1237.19367179777</v>
+      </c>
+      <c r="D9" s="10">
+        <f>MIN(C8,C9)</f>
+        <v>937.358386360928</v>
+      </c>
+      <c r="E9" s="10">
+        <f>MAX(B9,0)</f>
+        <v>299.835285436841</v>
+      </c>
+      <c r="F9" s="10">
+        <f>MAX(-B9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="10"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="24">
+        <f>Valuation!$C$7</f>
+        <v>4402.28172192655</v>
+      </c>
+      <c r="C10" s="10">
+        <f>C9+B10</f>
+        <v>5639.47539372432</v>
+      </c>
+      <c r="D10" s="10">
+        <f>MIN(C9,C10)</f>
+        <v>1237.19367179777</v>
+      </c>
+      <c r="E10" s="10">
+        <f>MAX(B10,0)</f>
+        <v>4402.28172192655</v>
+      </c>
+      <c r="F10" s="10">
+        <f>MAX(-B10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="10">
+        <f>C10</f>
+        <v>5639.47539372432</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="21">
+        <f>C11</f>
+        <v>5639.47539372432</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" s="12">
+        <v>2.32</v>
+      </c>
+      <c r="C38" s="12">
+        <v>5.96</v>
+      </c>
+      <c r="D38" s="23">
+        <f>C38-B38</f>
+        <v>3.64</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" s="12">
+        <v>2.14</v>
+      </c>
+      <c r="C39" s="12">
+        <v>5.78</v>
+      </c>
+      <c r="D39" s="23">
+        <f>C39-B39</f>
+        <v>3.64</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B40" s="12">
+        <v>1.82</v>
+      </c>
+      <c r="C40" s="12">
+        <v>4.57</v>
+      </c>
+      <c r="D40" s="23">
+        <f>C40-B40</f>
+        <v>2.75</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B41" s="12">
+        <v>5.68</v>
+      </c>
+      <c r="C41" s="12">
+        <v>5.699999999999999</v>
+      </c>
+      <c r="D41" s="23">
+        <f>C41-B41</f>
+        <v>0.0199999999999996</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="23">
+        <f>F42-ABS(F42)*G42</f>
+        <v>3.77355616459697</v>
+      </c>
+      <c r="C42" s="23">
+        <f>F42+ABS(F42)*G42</f>
+        <v>3.81148135218086</v>
+      </c>
+      <c r="D42" s="23">
+        <f>C42-B42</f>
+        <v>0.0379251875838893</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F42" s="25">
+        <f>Valuation!$C$11</f>
+        <v>3.79251875838892</v>
+      </c>
+      <c r="G42" s="26">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;A&amp;R&amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="34" max="16383" man="1"/>
+  </rowBreaks>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
@@ -1894,88 +3257,120 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="25">
+        <v>117</v>
+      </c>
+      <c r="B2" s="27">
         <f>Model!$G$16-Inputs!$C$21</f>
         <v>0</v>
       </c>
-      <c r="C2" s="26">
+      <c r="C2" s="28">
         <v>0.001</v>
       </c>
-      <c r="D2" s="27">
+      <c r="D2" s="29">
         <f>IF(ABS(B2)&lt;=C2,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="27">
-        <f>IF(Inputs!$C$17&gt;Inputs!$C$22,1,0)</f>
+        <v>118</v>
+      </c>
+      <c r="B3" s="29">
+        <f>IF(Inputs!$C$22&lt;Inputs!$C$17,1,0)</f>
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="27">
+        <v>119</v>
+      </c>
+      <c r="D3" s="29">
         <f>B3</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4" s="25">
+        <v>120</v>
+      </c>
+      <c r="B4" s="29">
+        <f>IF(MIN(Model!$C$14:$G$14)&gt;=0,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D4" s="29">
+        <f>B4</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="27">
         <f>Valuation!$C$10-SUM(Model!$C$22:$G$22)-Valuation!$C$7</f>
         <v>0</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C5" s="28">
         <v>0.001</v>
       </c>
-      <c r="D4" s="27">
-        <f>IF(ABS(B4)&lt;=C4,1,0)</f>
+      <c r="D5" s="29">
+        <f>IF(ABS(B5)&lt;=C5,1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" s="25">
+    <row r="6" spans="1:4">
+      <c r="A6" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="27">
         <f>Model!$G$7-(Inputs!$C$19+4)</f>
         <v>0</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C6" s="28">
         <v>0.001</v>
       </c>
-      <c r="D5" s="27">
-        <f>IF(ABS(B5)&lt;=C5,1,0)</f>
+      <c r="D6" s="29">
+        <f>IF(ABS(B6)&lt;=C6,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="28">
-        <f>IF(SUM(D2:D5)=4,1,0)</f>
+      <c r="A7" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="27">
+        <f>Charts!$G$11-Charts!$B$5-SUM(Charts!$B$6:Charts!$B$10)</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="28">
+        <v>0.001</v>
+      </c>
+      <c r="D7" s="29">
+        <f>IF(ABS(B7)&lt;=C7,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="30">
+        <f>IF(SUM(D2:D7)=COUNT(D2:D7),1,0)</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
excel-modeling: measured Google Sheets conversion, discount factor format
Uploaded probe workbooks through the Drive connector and read back what Sheets
computed. Defined names, cross-sheet lookups, _xlfn XLOOKUP/IFS/TEXTJOIN/MAXIFS,
CSE arrays, XNPV, date serials and number formats all survive; the full Jordan
model reproduces the local result (DCF $5,639m, $3.79 per share, master check
passing). The iterative-calc flag is not carried over (circular model shows
#REF!), What-If data tables flatten to cached values silently, and
_xlfn._xlws.SORT gives #NAME?. Structure (validation, charts, comments,
sparklines) cannot be inspected with the Drive connector alone. Upload limits
and the probe builder (tests/gsheets_lite.py) are documented.

Jordan workbook: discount factors now display to three decimals (was 0.0x).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFKfBcMnBcfuRQys4LRjyK
</commit_message>
<xml_diff>
--- a/data/valuation/jordan_valuation.xlsx
+++ b/data/valuation/jordan_valuation.xlsx
@@ -366,7 +366,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="143">
   <si>
     <t>Inputs</t>
   </si>
@@ -567,6 +567,9 @@
   </si>
   <si>
     <t>Discount factor</t>
+  </si>
+  <si>
+    <t>factor</t>
   </si>
   <si>
     <t>PV of free cash flow</t>
@@ -798,16 +801,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="@"/>
     <numFmt numFmtId="165" formatCode="#,##0_);(#,##0);&quot;-&quot;_)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00_);($#,##0.00);&quot;-&quot;_)"/>
     <numFmt numFmtId="167" formatCode="0.0%_);(0.0%);&quot;-&quot;_)"/>
     <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="#,##0.000000"/>
-    <numFmt numFmtId="172" formatCode="0.000000"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="172" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="173" formatCode="0.000000"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -927,13 +931,13 @@
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="173" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -1881,17 +1885,17 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B4" s="1" t="str">
         <f>IF(MasterCheck=1,"OK: all checks pass","ERROR: see Checks sheet")</f>
@@ -1900,44 +1904,44 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1945,7 +1949,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1953,23 +1957,23 @@
         <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2725,7 +2729,7 @@
         <v>66</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="C21" s="22">
         <f>1/(1+Inputs!$C$17)^C8</f>
@@ -2750,7 +2754,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>16</v>
@@ -2802,7 +2806,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2821,12 +2825,12 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>16</v>
@@ -2838,7 +2842,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>16</v>
@@ -2850,7 +2854,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>16</v>
@@ -2862,12 +2866,12 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>16</v>
@@ -2879,7 +2883,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>16</v>
@@ -2891,7 +2895,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>21</v>
@@ -2903,7 +2907,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>27</v>
@@ -2915,7 +2919,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>27</v>
@@ -2927,12 +2931,12 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>16</v>
@@ -2944,7 +2948,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>21</v>
@@ -2956,7 +2960,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>27</v>
@@ -2990,40 +2994,40 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>5</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" s="24">
         <f>Model!$C$22</f>
@@ -3043,7 +3047,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B6" s="24">
         <f>Model!$D$22</f>
@@ -3069,7 +3073,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B7" s="24">
         <f>Model!$E$22</f>
@@ -3095,7 +3099,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B8" s="24">
         <f>Model!$F$22</f>
@@ -3121,7 +3125,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B9" s="24">
         <f>Model!$G$22</f>
@@ -3147,7 +3151,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B10" s="24">
         <f>Valuation!$C$7</f>
@@ -3173,7 +3177,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C11" s="10">
         <f>C10</f>
@@ -3189,34 +3193,34 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B38" s="12">
         <v>2.32</v>
@@ -3229,12 +3233,12 @@
         <v>3.64</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B39" s="12">
         <v>2.14</v>
@@ -3247,12 +3251,12 @@
         <v>3.64</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B40" s="12">
         <v>1.82</v>
@@ -3265,12 +3269,12 @@
         <v>2.75</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B41" s="12">
         <v>5.68</v>
@@ -3283,12 +3287,12 @@
         <v>0.0199999999999996</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B42" s="23">
         <f>F42-ABS(F42)*G42</f>
@@ -3303,7 +3307,7 @@
         <v>0.0379251875838893</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F42" s="25">
         <f>Valuation!$C$11</f>
@@ -3315,7 +3319,7 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3343,21 +3347,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B2" s="27">
         <f>Model!$G$16-Inputs!$C$21</f>
@@ -3373,14 +3377,14 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B3" s="29">
         <f>IF(Inputs!$C$22&lt;Inputs!$C$17,1,0)</f>
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D3" s="29">
         <f>B3</f>
@@ -3389,14 +3393,14 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="29">
         <f>IF(MIN(Model!$C$14:$G$14)&gt;=0,1,0)</f>
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D4" s="29">
         <f>B4</f>
@@ -3405,7 +3409,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="27">
         <f>Valuation!$C$10-SUM(Model!$C$22:$G$22)-Valuation!$C$7</f>
@@ -3421,7 +3425,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="27">
         <f>Model!$G$7-(Inputs!$C$19+MAX(Model!$C$5:$G$5)-1)</f>
@@ -3437,7 +3441,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B7" s="27">
         <f>Charts!$G$11-Charts!$B$5-SUM(Charts!$B$6:$B$10)</f>
@@ -3453,7 +3457,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D9" s="30">
         <f>IF(SUM(D2:D7)=COUNT(D2:D7),1,0)</f>

</xml_diff>